<commit_message>
Actualizo todos los archivos
</commit_message>
<xml_diff>
--- a/casos_prueba_impuestos_codigo_limpio1.xlsx
+++ b/casos_prueba_impuestos_codigo_limpio1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dda7ef9302379344/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jp\OneDrive - Universidad de Medellin\Escritorio\Calculadora_Impuestos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B59A7CAF-0BFA-4FE1-A29E-C02C4DDAEDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ADAF835-EE43-42D1-90B8-0E291B1C20F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos Prueba Impuestos" sheetId="2" r:id="rId1"/>
@@ -90,12 +90,6 @@
     <t>Casos Extraordinarios</t>
   </si>
   <si>
-    <t>Alto Ejecutivo</t>
-  </si>
-  <si>
-    <t>Salario Mínimo</t>
-  </si>
-  <si>
     <t>Casos de Error</t>
   </si>
   <si>
@@ -136,6 +130,12 @@
   </si>
   <si>
     <t>ERROR: Los ingresos deben ser un valor numérico</t>
+  </si>
+  <si>
+    <t>Casos Extraordinarios 1</t>
+  </si>
+  <si>
+    <t>Casos Extraordinario 2</t>
   </si>
 </sst>
 </file>
@@ -221,12 +221,6 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -241,6 +235,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -507,7 +507,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -520,114 +520,114 @@
     <col min="11" max="11" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-    </row>
-    <row r="3" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+    </row>
+    <row r="3" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1" t="s">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+    </row>
+    <row r="4" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" ht="135.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" ht="179.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <v>80000000</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="4">
         <v>10000000</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>6400000</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
         <v>3200000</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="3">
         <v>2</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="3">
         <v>1</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="3">
         <f>MAX(0, B6-C6-D6-E6)</f>
         <v>60400000</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="3">
         <f>IF((H6/52374)&lt;=1090, 0,
 IF((H6/52374)&lt;=1700, ROUND(((H6/52374)-1090)*0.19*52374,0),
 IF((H6/52374)&lt;=4100, ROUND((116 + ((H6/52374)-1700)*0.28)*52374,0),
@@ -637,11 +637,11 @@
 ROUND((10352 + ((H6/52374)-31000)*0.39)*52374,0)))))))</f>
         <v>629345</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="3">
         <f>IF(B6&gt;0, (I6/B6)*100, 0)</f>
         <v>0.78668125</v>
       </c>
-      <c r="K6" s="5" t="str">
+      <c r="K6" s="3" t="str">
         <f>A6&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Ingresos: $"&amp;TEXT(B6,"#,##0")&amp;CHAR(10)&amp;"- Deducciones: $"&amp;TEXT(C6,"#,##0")&amp;CHAR(10)&amp;"- Pensión: $"&amp;TEXT(D6,"#,##0")&amp;CHAR(10)&amp;"- Salud: $"&amp;TEXT(E6,"#,##0")&amp;CHAR(10)&amp;"- Dependientes: "&amp;F6&amp;CHAR(10)&amp;"Salidas:"&amp;CHAR(10)&amp;"- Impuesto: $"&amp;TEXT(ROUND(I6,0),"#,##0")&amp;CHAR(10)&amp;"- Tasa: "&amp;TEXT(J6,"0.00")&amp;"%"</f>
         <v>Caso Normal 1
 Entradas:
@@ -655,33 +655,33 @@
 - Tasa: 001%</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="135.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:11" ht="164.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="4">
         <v>150000000</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="4">
         <v>20000000</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>12000000</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="4">
         <v>6000000</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="3">
         <v>1</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="3">
         <v>0</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="3">
         <f>MAX(0, B7-C7-D7-E7)</f>
         <v>112000000</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="3">
         <f>IF((H7/52374)&lt;=1090, 0,
 IF((H7/52374)&lt;=1700, ROUND(((H7/52374)-1090)*0.19*52374,0),
 IF((H7/52374)&lt;=4100, ROUND((116 + ((H7/52374)-1700)*0.28)*52374,0),
@@ -691,11 +691,11 @@
 ROUND((10352 + ((H7/52374)-31000)*0.39)*52374,0)))))))</f>
         <v>12505360</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="3">
         <f>IF(B7&gt;0, (I7/B7)*100, 0)</f>
         <v>8.3369066666666676</v>
       </c>
-      <c r="K7" s="5" t="str">
+      <c r="K7" s="3" t="str">
         <f>A7&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Ingresos: $"&amp;TEXT(B7,"#,##0")&amp;CHAR(10)&amp;"- Deducciones: $"&amp;TEXT(C7,"#,##0")&amp;CHAR(10)&amp;"- Pensión: $"&amp;TEXT(D7,"#,##0")&amp;CHAR(10)&amp;"- Salud: $"&amp;TEXT(E7,"#,##0")&amp;CHAR(10)&amp;"- Dependientes: "&amp;F7&amp;CHAR(10)&amp;"Salidas:"&amp;CHAR(10)&amp;"- Impuesto: $"&amp;TEXT(ROUND(I7,0),"#,##0")&amp;CHAR(10)&amp;"- Tasa: "&amp;TEXT(J7,"0.00")&amp;"%"</f>
         <v>Caso Normal 2
 Entradas:
@@ -709,61 +709,61 @@
 - Tasa: 008%</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-    </row>
-    <row r="9" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-    </row>
-    <row r="10" spans="1:11" ht="135.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="6">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" ht="135.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="4">
         <v>600000000</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="4">
         <v>60000000</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>48000000</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <v>24000000</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="3">
         <v>4</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="3">
         <v>1</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="3">
         <f>MAX(0, B10-C10-D10-E10)</f>
         <v>468000000</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="3">
         <f>IF((H10/52374)&lt;=1090, 0,
 IF((H10/52374)&lt;=1700, ROUND(((H10/52374)-1090)*0.19*52374,0),
 IF((H10/52374)&lt;=4100, ROUND((116 + ((H10/52374)-1700)*0.28)*52374,0),
@@ -773,13 +773,13 @@
 ROUND((10352 + ((H10/52374)-31000)*0.39)*52374,0)))))))</f>
         <v>125121801</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="3">
         <f>IF(B10&gt;0, (I10/B10)*100, 0)</f>
         <v>20.853633499999997</v>
       </c>
-      <c r="K10" s="5" t="str">
+      <c r="K10" s="3" t="str">
         <f>A10&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Ingresos: $"&amp;TEXT(B10,"#,##0")&amp;CHAR(10)&amp;"- Deducciones: $"&amp;TEXT(C10,"#,##0")&amp;CHAR(10)&amp;"- Pensión: $"&amp;TEXT(D10,"#,##0")&amp;CHAR(10)&amp;"- Salud: $"&amp;TEXT(E10,"#,##0")&amp;CHAR(10)&amp;"- Dependientes: "&amp;F10&amp;CHAR(10)&amp;"Salidas:"&amp;CHAR(10)&amp;"- Impuesto: $"&amp;TEXT(ROUND(I10,0),"#,##0")&amp;CHAR(10)&amp;"- Tasa: "&amp;TEXT(J10,"0.00")&amp;"%"</f>
-        <v>Alto Ejecutivo
+        <v>Casos Extraordinarios 1
 Entradas:
 - Ingresos: $600000000,0
 - Deducciones: $60000000,0
@@ -791,33 +791,33 @@
 - Tasa: 021%</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="135.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="6">
+    <row r="11" spans="1:11" ht="135.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="4">
         <v>15000000</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="4">
         <v>0</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>1200000</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="4">
         <v>600000</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="3">
         <v>0</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="3">
         <v>0</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="3">
         <f>MAX(0, B11-C11-D11-E11)</f>
         <v>13200000</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="3">
         <f>IF((H11/52374)&lt;=1090, 0,
 IF((H11/52374)&lt;=1700, ROUND(((H11/52374)-1090)*0.19*52374,0),
 IF((H11/52374)&lt;=4100, ROUND((116 + ((H11/52374)-1700)*0.28)*52374,0),
@@ -827,13 +827,13 @@
 ROUND((10352 + ((H11/52374)-31000)*0.39)*52374,0)))))))</f>
         <v>0</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="3">
         <f>IF(B11&gt;0, (I11/B11)*100, 0)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="5" t="str">
+      <c r="K11" s="3" t="str">
         <f>A11&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Ingresos: $"&amp;TEXT(B11,"#,##0")&amp;CHAR(10)&amp;"- Deducciones: $"&amp;TEXT(C11,"#,##0")&amp;CHAR(10)&amp;"- Pensión: $"&amp;TEXT(D11,"#,##0")&amp;CHAR(10)&amp;"- Salud: $"&amp;TEXT(E11,"#,##0")&amp;CHAR(10)&amp;"- Dependientes: "&amp;F11&amp;CHAR(10)&amp;"Salidas:"&amp;CHAR(10)&amp;"- Impuesto: $"&amp;TEXT(ROUND(I11,0),"#,##0")&amp;CHAR(10)&amp;"- Tasa: "&amp;TEXT(J11,"0.00")&amp;"%"</f>
-        <v>Salario Mínimo
+        <v>Casos Extraordinario 2
 Entradas:
 - Ingresos: $15000000,0
 - Deducciones: $,0
@@ -845,66 +845,66 @@
 - Tasa: 000%</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-    </row>
-    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
+    <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="4">
+        <v>-50000000</v>
+      </c>
+      <c r="C14" s="4">
+        <v>5000000</v>
+      </c>
+      <c r="D14" s="4">
+        <v>4000000</v>
+      </c>
+      <c r="E14" s="4">
+        <v>2000000</v>
+      </c>
+      <c r="F14" s="3">
+        <v>1</v>
+      </c>
+      <c r="G14" s="3">
+        <v>1</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-    </row>
-    <row r="14" spans="1:11" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
+      <c r="I14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="6">
-        <v>-50000000</v>
-      </c>
-      <c r="C14" s="6">
-        <v>5000000</v>
-      </c>
-      <c r="D14" s="6">
-        <v>4000000</v>
-      </c>
-      <c r="E14" s="6">
-        <v>2000000</v>
-      </c>
-      <c r="F14" s="5">
-        <v>1</v>
-      </c>
-      <c r="G14" s="5">
-        <v>1</v>
-      </c>
-      <c r="H14" s="5" t="s">
+      <c r="J14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I14" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="K14" s="5" t="str">
+      <c r="K14" s="3" t="str">
         <f>A14&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Ingresos: $"&amp;TEXT(B14,"#,##0")&amp;CHAR(10)&amp;"Error: Los ingresos deben ser mayores o iguales a cero"</f>
         <v>Error: Ingresos Negativos
 Entradas:
@@ -912,39 +912,39 @@
 Error: Los ingresos deben ser mayores o iguales a cero</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="68.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="6">
+    <row r="15" spans="1:11" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="4">
         <v>50000000</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="4">
         <v>60000000</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="4">
         <v>4000000</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="4">
         <v>2000000</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="3">
         <v>2</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="3">
         <v>0</v>
       </c>
-      <c r="H15" s="5" t="str">
+      <c r="H15" s="3" t="str">
         <f>IF(C15&gt;B15, "ERROR", MAX(0, B15-C15-D15-E15))</f>
         <v>ERROR</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="J15" s="5" t="s">
+      <c r="I15" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K15" s="5" t="str">
+      <c r="J15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" s="3" t="str">
         <f>A15&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Ingresos: $"&amp;TEXT(B15,"#,##0")&amp;CHAR(10)&amp;"- Deducciones: $"&amp;TEXT(C15,"#,##0")&amp;CHAR(10)&amp;"Error: Las deducciones superan los ingresos"</f>
         <v>Error: Deducciones Excesivas
 Entradas:
@@ -953,38 +953,38 @@
 Error: Las deducciones superan los ingresos</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="6">
+    <row r="16" spans="1:11" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="4">
         <v>80000000</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="4">
         <v>10000000</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="4">
         <v>6400000</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="4">
         <v>3200000</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="3">
         <v>-2</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="3">
         <v>1</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="H16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="K16" s="5" t="str">
+      <c r="K16" s="3" t="str">
         <f>A16&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Dependientes: "&amp;F16&amp;CHAR(10)&amp;"Error: Los dependientes no pueden ser negativos"</f>
         <v>Error: Dependientes Negativos
 Entradas:
@@ -992,73 +992,73 @@
 Error: Los dependientes no pueden ser negativos</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="6">
+    <row r="17" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="4">
         <v>8000000</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="4">
         <v>5000000</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="4">
         <v>2500000</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="3">
         <v>1</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="3">
         <v>1</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I17" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="K17" s="5" t="str">
+      <c r="K17" s="3" t="str">
         <f>A17&amp;CHAR(10)&amp;"Error: El campo de ingresos está vacío y es obligatorio"</f>
         <v>Error: Campo Vacío
 Error: El campo de ingresos está vacío y es obligatorio</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="1:11" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="4">
+        <v>10000000</v>
+      </c>
+      <c r="D18" s="4">
+        <v>8000000</v>
+      </c>
+      <c r="E18" s="4">
+        <v>4000000</v>
+      </c>
+      <c r="F18" s="3">
+        <v>3</v>
+      </c>
+      <c r="G18" s="3">
+        <v>1</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I18" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="6">
-        <v>10000000</v>
-      </c>
-      <c r="D18" s="6">
-        <v>8000000</v>
-      </c>
-      <c r="E18" s="6">
-        <v>4000000</v>
-      </c>
-      <c r="F18" s="5">
-        <v>3</v>
-      </c>
-      <c r="G18" s="5">
-        <v>1</v>
-      </c>
-      <c r="H18" s="5" t="s">
+      <c r="J18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="K18" s="5" t="str">
+      <c r="K18" s="3" t="str">
         <f>A18&amp;CHAR(10)&amp;"Entradas:"&amp;CHAR(10)&amp;"- Ingresos: "&amp;B18&amp;CHAR(10)&amp;"Error: El valor debe ser numérico"</f>
         <v>Error: Tipo Dato Incorrecto
 Entradas:

</xml_diff>

<commit_message>
Cambios de en lógica y pruebas
</commit_message>
<xml_diff>
--- a/casos_prueba_impuestos_codigo_limpio1.xlsx
+++ b/casos_prueba_impuestos_codigo_limpio1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jp\OneDrive - Universidad de Medellin\Escritorio\Calculadora_Impuestos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ADAF835-EE43-42D1-90B8-0E291B1C20F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2B89A6-4803-4DFE-9B30-B9C3ADFE5794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3660" yWindow="3540" windowWidth="17280" windowHeight="9420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos Prueba Impuestos" sheetId="2" r:id="rId1"/>

</xml_diff>